<commit_message>
Unhide Demand Models and exFactory Demand Model sheets
</commit_message>
<xml_diff>
--- a/Cardamyst Affordability Model - Final.xlsx
+++ b/Cardamyst Affordability Model - Final.xlsx
@@ -10,8 +10,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="2" state="hidden" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Demand Models" sheetId="5" state="hidden" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="exFactory Demand Model" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Demand Models" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="exFactory Demand Model" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accruals" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Charts" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>

</xml_diff>

<commit_message>
Move ExFactory to Demand tab, delete separate sheet
Demand tab now has all demand data in one place:
- Scenario 1: Original Base Model (rows 10-14)
- Scenario 2: BOD Demand (rows 16-22)
- ExFactory (rows 27-34): Script Demand, MOH Target, Beg/End Balance, ExFactory Units

Accruals updated to reference Demand!row34 for ExFactory units
</commit_message>
<xml_diff>
--- a/Cardamyst Affordability Model - Final.xlsx
+++ b/Cardamyst Affordability Model - Final.xlsx
@@ -9,10 +9,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="START HERE" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Demand" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ExFactory" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accruals" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accruals" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -33,7 +32,7 @@
     <numFmt numFmtId="172" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="173" formatCode="[$-409]mmm\-yy;@"/>
   </numFmts>
-  <fonts count="36">
+  <fonts count="37">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -251,6 +250,12 @@
       <color rgb="00E31D93"/>
       <sz val="14"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00E31D93"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="19">
     <fill>
@@ -361,7 +366,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -413,6 +418,20 @@
         <color rgb="00172852"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0"/>
@@ -421,7 +440,7 @@
     <xf numFmtId="43" fontId="20" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="25" fillId="11" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="110">
+  <cellXfs count="118">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -552,6 +571,20 @@
     <xf numFmtId="172" fontId="0" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="27" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="33" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="29" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="29" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="29" fillId="14" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="36" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3741,7 +3774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O29"/>
+  <dimension ref="A1:O34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" bestFit="1" customWidth="1" style="74" min="1" max="1"/>
@@ -3790,8 +3823,6 @@
       </c>
     </row>
     <row r="4" ht="23.25" customHeight="1" s="74"/>
-    <row r="5"/>
-    <row r="6"/>
     <row r="7" ht="15.75" customHeight="1" s="74">
       <c r="A7" s="84" t="inlineStr">
         <is>
@@ -3800,7 +3831,6 @@
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1" s="74"/>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="103" t="inlineStr">
         <is>
@@ -3948,15 +3978,6 @@
         <is>
           <t>TRx Forecast (Covered Commercial)</t>
         </is>
-      </c>
-      <c r="C13" s="86" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="86" t="n">
-        <v>50.23</v>
-      </c>
-      <c r="E13" s="86" t="n">
-        <v>83.78</v>
       </c>
       <c r="F13" s="86" t="n">
         <v>131.82</v>
@@ -4415,18 +4436,35 @@
         <v/>
       </c>
     </row>
-    <row r="23"/>
     <row r="24" ht="23.25" customHeight="1" s="74"/>
     <row r="25" ht="15.75" customHeight="1" s="74"/>
-    <row r="26"/>
     <row r="27">
-      <c r="A27" s="84" t="inlineStr">
-        <is>
-          <t>Ex-Factory Demand Scenarios</t>
-        </is>
-      </c>
+      <c r="A27" s="110" t="inlineStr">
+        <is>
+          <t>EXFACTORY DEMAND (Channel Inventory)</t>
+        </is>
+      </c>
+      <c r="B27" s="109" t="n"/>
+      <c r="C27" s="109" t="n"/>
+      <c r="D27" s="109" t="n"/>
+      <c r="E27" s="109" t="n"/>
+      <c r="F27" s="109" t="n"/>
+      <c r="G27" s="109" t="n"/>
+      <c r="H27" s="109" t="n"/>
+      <c r="I27" s="109" t="n"/>
+      <c r="J27" s="109" t="n"/>
+      <c r="K27" s="109" t="n"/>
+      <c r="L27" s="109" t="n"/>
+      <c r="M27" s="109" t="n"/>
+      <c r="N27" s="109" t="n"/>
+      <c r="O27" s="109" t="n"/>
     </row>
     <row r="28">
+      <c r="A28" s="98" t="inlineStr">
+        <is>
+          <t>→ ExFactory = units shipped to wholesalers for revenue recognition</t>
+        </is>
+      </c>
       <c r="C28" s="80" t="inlineStr">
         <is>
           <t>Jan</t>
@@ -4494,10 +4532,329 @@
       </c>
     </row>
     <row r="29">
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Beginning of Month Channel Balance</t>
-        </is>
+      <c r="A29" s="111" t="inlineStr"/>
+      <c r="B29" s="111" t="inlineStr"/>
+      <c r="C29" s="111" t="inlineStr">
+        <is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="D29" s="111" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="E29" s="111" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="F29" s="111" t="inlineStr">
+        <is>
+          <t>Apr</t>
+        </is>
+      </c>
+      <c r="G29" s="111" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="H29" s="111" t="inlineStr">
+        <is>
+          <t>Jun</t>
+        </is>
+      </c>
+      <c r="I29" s="111" t="inlineStr">
+        <is>
+          <t>Jul</t>
+        </is>
+      </c>
+      <c r="J29" s="111" t="inlineStr">
+        <is>
+          <t>Aug</t>
+        </is>
+      </c>
+      <c r="K29" s="111" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="L29" s="111" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="M29" s="111" t="inlineStr">
+        <is>
+          <t>Nov</t>
+        </is>
+      </c>
+      <c r="N29" s="111" t="inlineStr">
+        <is>
+          <t>Dec</t>
+        </is>
+      </c>
+      <c r="O29" s="111" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="112" t="inlineStr">
+        <is>
+          <t>Script Demand (Rx)</t>
+        </is>
+      </c>
+      <c r="C30" s="113" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="113" t="n">
+        <v>130</v>
+      </c>
+      <c r="E30" s="113" t="n">
+        <v>246</v>
+      </c>
+      <c r="F30" s="113" t="n">
+        <v>445</v>
+      </c>
+      <c r="G30" s="113" t="n">
+        <v>827</v>
+      </c>
+      <c r="H30" s="113" t="n">
+        <v>1273</v>
+      </c>
+      <c r="I30" s="113" t="n">
+        <v>2290</v>
+      </c>
+      <c r="J30" s="113" t="n">
+        <v>3028</v>
+      </c>
+      <c r="K30" s="113" t="n">
+        <v>3919</v>
+      </c>
+      <c r="L30" s="113" t="n">
+        <v>4772</v>
+      </c>
+      <c r="M30" s="113" t="n">
+        <v>5745</v>
+      </c>
+      <c r="N30" s="113" t="n">
+        <v>6813</v>
+      </c>
+      <c r="O30" s="114">
+        <f>SUM(C30:N30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="112" t="inlineStr">
+        <is>
+          <t>MOH Target</t>
+        </is>
+      </c>
+      <c r="C31" s="115" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="115" t="n">
+        <v>2</v>
+      </c>
+      <c r="E31" s="115" t="n">
+        <v>2</v>
+      </c>
+      <c r="F31" s="115" t="n">
+        <v>2</v>
+      </c>
+      <c r="G31" s="115" t="n">
+        <v>2</v>
+      </c>
+      <c r="H31" s="115" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="I31" s="115" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="J31" s="115" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="K31" s="115" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="L31" s="115" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="M31" s="115" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="N31" s="115" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="112" t="inlineStr">
+        <is>
+          <t>Beg of Month Balance</t>
+        </is>
+      </c>
+      <c r="C32" s="114" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="113">
+        <f>C33</f>
+        <v/>
+      </c>
+      <c r="E32" s="113">
+        <f>D33</f>
+        <v/>
+      </c>
+      <c r="F32" s="113">
+        <f>E33</f>
+        <v/>
+      </c>
+      <c r="G32" s="113">
+        <f>F33</f>
+        <v/>
+      </c>
+      <c r="H32" s="113">
+        <f>G33</f>
+        <v/>
+      </c>
+      <c r="I32" s="113">
+        <f>H33</f>
+        <v/>
+      </c>
+      <c r="J32" s="113">
+        <f>I33</f>
+        <v/>
+      </c>
+      <c r="K32" s="113">
+        <f>J33</f>
+        <v/>
+      </c>
+      <c r="L32" s="113">
+        <f>K33</f>
+        <v/>
+      </c>
+      <c r="M32" s="113">
+        <f>L33</f>
+        <v/>
+      </c>
+      <c r="N32" s="113">
+        <f>M33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="112" t="inlineStr">
+        <is>
+          <t>End of Month Balance</t>
+        </is>
+      </c>
+      <c r="C33" s="113">
+        <f>C30*C31</f>
+        <v/>
+      </c>
+      <c r="D33" s="113">
+        <f>D30*D31</f>
+        <v/>
+      </c>
+      <c r="E33" s="113">
+        <f>E30*E31</f>
+        <v/>
+      </c>
+      <c r="F33" s="113">
+        <f>F30*F31</f>
+        <v/>
+      </c>
+      <c r="G33" s="113">
+        <f>G30*G31</f>
+        <v/>
+      </c>
+      <c r="H33" s="113">
+        <f>H30*H31</f>
+        <v/>
+      </c>
+      <c r="I33" s="113">
+        <f>I30*I31</f>
+        <v/>
+      </c>
+      <c r="J33" s="113">
+        <f>J30*J31</f>
+        <v/>
+      </c>
+      <c r="K33" s="113">
+        <f>K30*K31</f>
+        <v/>
+      </c>
+      <c r="L33" s="113">
+        <f>L30*L31</f>
+        <v/>
+      </c>
+      <c r="M33" s="113">
+        <f>M30*M31</f>
+        <v/>
+      </c>
+      <c r="N33" s="113">
+        <f>N30*N31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="116" t="inlineStr">
+        <is>
+          <t>ExFactory Units</t>
+        </is>
+      </c>
+      <c r="C34" s="114" t="n">
+        <v>474</v>
+      </c>
+      <c r="D34" s="113">
+        <f>IF(D32-D30&gt;D33,0,D33-D32+D30)</f>
+        <v/>
+      </c>
+      <c r="E34" s="113">
+        <f>IF(E32-E30&gt;E33,0,E33-E32+E30)</f>
+        <v/>
+      </c>
+      <c r="F34" s="113">
+        <f>IF(F32-F30&gt;F33,0,F33-F32+F30)</f>
+        <v/>
+      </c>
+      <c r="G34" s="113">
+        <f>IF(G32-G30&gt;G33,0,G33-G32+G30)</f>
+        <v/>
+      </c>
+      <c r="H34" s="113">
+        <f>IF(H32-H30&gt;H33,0,H33-H32+H30)</f>
+        <v/>
+      </c>
+      <c r="I34" s="113">
+        <f>IF(I32-I30&gt;I33,0,I33-I32+I30)</f>
+        <v/>
+      </c>
+      <c r="J34" s="113">
+        <f>IF(J32-J30&gt;J33,0,J33-J32+J30)</f>
+        <v/>
+      </c>
+      <c r="K34" s="113">
+        <f>IF(K32-K30&gt;K33,0,K33-K32+K30)</f>
+        <v/>
+      </c>
+      <c r="L34" s="113">
+        <f>IF(L32-L30&gt;L33,0,L33-L32+L30)</f>
+        <v/>
+      </c>
+      <c r="M34" s="113">
+        <f>IF(M32-M30&gt;M33,0,M33-M32+M30)</f>
+        <v/>
+      </c>
+      <c r="N34" s="113">
+        <f>IF(N32-N30&gt;N33,0,N33-N32+N30)</f>
+        <v/>
+      </c>
+      <c r="O34" s="117">
+        <f>SUM(C34:N34)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -4513,635 +4870,6 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J42"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="15" bestFit="1" customWidth="1" style="74" min="2" max="2"/>
-    <col width="28" customWidth="1" style="74" min="3" max="3"/>
-    <col width="28" customWidth="1" style="74" min="4" max="4"/>
-    <col width="25" customWidth="1" style="74" min="5" max="5"/>
-    <col width="15" customWidth="1" style="74" min="6" max="6"/>
-    <col width="28" customWidth="1" style="74" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="B1" s="108" t="inlineStr">
-        <is>
-          <t>EXFACTORY DEMAND - Channel inventory model for revenue recognition</t>
-        </is>
-      </c>
-      <c r="C1" s="109" t="n"/>
-      <c r="D1" s="109" t="n"/>
-      <c r="E1" s="109" t="n"/>
-      <c r="F1" s="109" t="n"/>
-      <c r="G1" s="109" t="n"/>
-      <c r="H1" s="109" t="n"/>
-      <c r="I1" s="109" t="n"/>
-      <c r="J1" s="109" t="n"/>
-    </row>
-    <row r="2" ht="30" customHeight="1" s="74">
-      <c r="B2" s="98" t="inlineStr">
-        <is>
-          <t>→ ExFactory units flow to Accruals tab for income statement GTN calculations</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="B3" s="64" t="n"/>
-      <c r="C3" s="65" t="inlineStr">
-        <is>
-          <t>Beg of month channel balance</t>
-        </is>
-      </c>
-      <c r="D3" s="65" t="inlineStr">
-        <is>
-          <t>Total Monthly Script Demand (Forecast)</t>
-        </is>
-      </c>
-      <c r="E3" s="65" t="inlineStr">
-        <is>
-          <t>End of month channel balance</t>
-        </is>
-      </c>
-      <c r="F3" s="65" t="inlineStr">
-        <is>
-          <t>MOH Assumption</t>
-        </is>
-      </c>
-      <c r="G3" s="65" t="inlineStr">
-        <is>
-          <t>Total Monthly exFact Demand (Forecast)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" s="64" t="n">
-        <v>46022</v>
-      </c>
-      <c r="C4" s="72" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" s="72" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" s="67">
-        <f>+C3-D3+G3</f>
-        <v/>
-      </c>
-      <c r="F4" s="72" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" s="72" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" s="64">
-        <f>EOMONTH(B3+1,0)</f>
-        <v/>
-      </c>
-      <c r="C5" s="67">
-        <f>E3</f>
-        <v/>
-      </c>
-      <c r="D5" s="72" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="67">
-        <f>+G4</f>
-        <v/>
-      </c>
-      <c r="F5" s="68" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="72" t="n">
-        <v>474</v>
-      </c>
-      <c r="J5" s="67" t="n"/>
-    </row>
-    <row r="6">
-      <c r="B6" s="64">
-        <f>EOMONTH(B4+1,0)</f>
-        <v/>
-      </c>
-      <c r="C6" s="67">
-        <f>+E4</f>
-        <v/>
-      </c>
-      <c r="D6" s="72" t="n">
-        <v>130</v>
-      </c>
-      <c r="E6" s="67">
-        <f>+F5*D5</f>
-        <v/>
-      </c>
-      <c r="F6" s="68" t="n">
-        <v>2</v>
-      </c>
-      <c r="G6" s="72">
-        <f>+IF(C5-D5&gt;E5,0,E5-C5+D5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="64">
-        <f>EOMONTH(B5+1,0)</f>
-        <v/>
-      </c>
-      <c r="C7" s="67">
-        <f>+E5</f>
-        <v/>
-      </c>
-      <c r="D7" s="72" t="n">
-        <v>246</v>
-      </c>
-      <c r="E7" s="67">
-        <f>+F6*D6</f>
-        <v/>
-      </c>
-      <c r="F7" s="68" t="n">
-        <v>2</v>
-      </c>
-      <c r="G7" s="72">
-        <f>+IF(C6-D6&gt;E6,0,E6-C6+D6)</f>
-        <v/>
-      </c>
-      <c r="H7" s="68" t="n"/>
-    </row>
-    <row r="8">
-      <c r="B8" s="64">
-        <f>EOMONTH(B6+1,0)</f>
-        <v/>
-      </c>
-      <c r="C8" s="67">
-        <f>+E6</f>
-        <v/>
-      </c>
-      <c r="D8" s="72" t="n">
-        <v>445</v>
-      </c>
-      <c r="E8" s="67">
-        <f>+F7*D7</f>
-        <v/>
-      </c>
-      <c r="F8" s="68" t="n">
-        <v>2</v>
-      </c>
-      <c r="G8" s="72">
-        <f>+IF(C7-D7&gt;E7,0,E7-C7+D7)</f>
-        <v/>
-      </c>
-      <c r="H8" s="68" t="n"/>
-    </row>
-    <row r="9">
-      <c r="B9" s="64">
-        <f>EOMONTH(B7+1,0)</f>
-        <v/>
-      </c>
-      <c r="C9" s="67">
-        <f>+E7</f>
-        <v/>
-      </c>
-      <c r="D9" s="72" t="n">
-        <v>827</v>
-      </c>
-      <c r="E9" s="67">
-        <f>+F8*D8</f>
-        <v/>
-      </c>
-      <c r="F9" s="68" t="n">
-        <v>2</v>
-      </c>
-      <c r="G9" s="72">
-        <f>+IF(C8-D8&gt;E8,0,E8-C8+D8)</f>
-        <v/>
-      </c>
-      <c r="H9" s="68" t="n"/>
-    </row>
-    <row r="10">
-      <c r="B10" s="64">
-        <f>EOMONTH(B8+1,0)</f>
-        <v/>
-      </c>
-      <c r="C10" s="67">
-        <f>+E8</f>
-        <v/>
-      </c>
-      <c r="D10" s="72" t="n">
-        <v>1273</v>
-      </c>
-      <c r="E10" s="67">
-        <f>+F9*D9</f>
-        <v/>
-      </c>
-      <c r="F10" s="68" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="G10" s="72">
-        <f>+IF(C9-D9&gt;E9,0,E9-C9+D9)</f>
-        <v/>
-      </c>
-      <c r="H10" s="68" t="n"/>
-    </row>
-    <row r="11">
-      <c r="B11" s="64">
-        <f>EOMONTH(B9+1,0)</f>
-        <v/>
-      </c>
-      <c r="C11" s="67">
-        <f>+E9</f>
-        <v/>
-      </c>
-      <c r="D11" s="72" t="n">
-        <v>2290</v>
-      </c>
-      <c r="E11" s="67">
-        <f>+F10*D10</f>
-        <v/>
-      </c>
-      <c r="F11" s="68" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="G11" s="72">
-        <f>+IF(C10-D10&gt;E10,0,E10-C10+D10)</f>
-        <v/>
-      </c>
-      <c r="H11" s="68" t="n"/>
-    </row>
-    <row r="12">
-      <c r="B12" s="64">
-        <f>EOMONTH(B10+1,0)</f>
-        <v/>
-      </c>
-      <c r="C12" s="67">
-        <f>+E10</f>
-        <v/>
-      </c>
-      <c r="D12" s="72" t="n">
-        <v>3028</v>
-      </c>
-      <c r="E12" s="67">
-        <f>+F11*D11</f>
-        <v/>
-      </c>
-      <c r="F12" s="68" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="G12" s="72">
-        <f>+IF(C11-D11&gt;E11,0,E11-C11+D11)</f>
-        <v/>
-      </c>
-      <c r="H12" s="68" t="n"/>
-    </row>
-    <row r="13">
-      <c r="B13" s="64">
-        <f>EOMONTH(B11+1,0)</f>
-        <v/>
-      </c>
-      <c r="C13" s="67">
-        <f>+E11</f>
-        <v/>
-      </c>
-      <c r="D13" s="72" t="n">
-        <v>3919</v>
-      </c>
-      <c r="E13" s="67">
-        <f>+F12*D12</f>
-        <v/>
-      </c>
-      <c r="F13" s="68" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="G13" s="72">
-        <f>+IF(C12-D12&gt;E12,0,E12-C12+D12)</f>
-        <v/>
-      </c>
-      <c r="H13" s="68" t="n"/>
-    </row>
-    <row r="14">
-      <c r="B14" s="64">
-        <f>EOMONTH(B12+1,0)</f>
-        <v/>
-      </c>
-      <c r="C14" s="67">
-        <f>+E12</f>
-        <v/>
-      </c>
-      <c r="D14" s="72" t="n">
-        <v>4772</v>
-      </c>
-      <c r="E14" s="67">
-        <f>+F13*D13</f>
-        <v/>
-      </c>
-      <c r="F14" s="68" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="G14" s="72">
-        <f>+IF(C13-D13&gt;E13,0,E13-C13+D13)</f>
-        <v/>
-      </c>
-      <c r="H14" s="68" t="n"/>
-    </row>
-    <row r="15">
-      <c r="B15" s="64">
-        <f>EOMONTH(B13+1,0)</f>
-        <v/>
-      </c>
-      <c r="C15" s="67">
-        <f>+E13</f>
-        <v/>
-      </c>
-      <c r="D15" s="72" t="n">
-        <v>5745</v>
-      </c>
-      <c r="E15" s="67">
-        <f>+F14*D14</f>
-        <v/>
-      </c>
-      <c r="F15" s="68" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="G15" s="72">
-        <f>+IF(C14-D14&gt;E14,0,E14-C14+D14)</f>
-        <v/>
-      </c>
-      <c r="H15" s="68" t="n"/>
-    </row>
-    <row r="16">
-      <c r="B16" s="64">
-        <f>EOMONTH(B14+1,0)</f>
-        <v/>
-      </c>
-      <c r="C16" s="67">
-        <f>+E14</f>
-        <v/>
-      </c>
-      <c r="D16" s="72" t="n">
-        <v>6813</v>
-      </c>
-      <c r="E16" s="67">
-        <f>+F15*D15</f>
-        <v/>
-      </c>
-      <c r="F16" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="G16" s="72">
-        <f>+IF(C15-D15&gt;E15,0,E15-C15+D15)</f>
-        <v/>
-      </c>
-      <c r="H16" s="68" t="n"/>
-    </row>
-    <row r="17">
-      <c r="B17" s="64">
-        <f>EOMONTH(B15+1,0)</f>
-        <v/>
-      </c>
-      <c r="C17" s="67">
-        <f>+E15</f>
-        <v/>
-      </c>
-      <c r="D17" s="67" t="n">
-        <v>8673</v>
-      </c>
-      <c r="E17" s="67">
-        <f>+F16*D16</f>
-        <v/>
-      </c>
-      <c r="F17" s="68" t="n">
-        <v>1</v>
-      </c>
-      <c r="G17" s="72">
-        <f>+IF(C16-D16&gt;E16,0,E16-C16+D16)</f>
-        <v/>
-      </c>
-      <c r="H17" s="68" t="n"/>
-    </row>
-    <row r="18">
-      <c r="B18" s="70" t="n"/>
-      <c r="C18" s="67" t="n"/>
-      <c r="D18" s="86" t="n"/>
-      <c r="E18" s="67" t="n"/>
-      <c r="F18" s="68" t="n"/>
-      <c r="G18" s="72" t="n"/>
-      <c r="H18" s="68" t="n"/>
-    </row>
-    <row r="19">
-      <c r="B19" s="70" t="n"/>
-      <c r="C19" s="67" t="n"/>
-      <c r="D19" s="86" t="n"/>
-      <c r="E19" s="67" t="n"/>
-      <c r="F19" s="68" t="n"/>
-      <c r="G19" s="72" t="n"/>
-      <c r="H19" s="68" t="n"/>
-    </row>
-    <row r="20">
-      <c r="B20" s="70" t="n"/>
-      <c r="C20" s="67" t="n"/>
-      <c r="D20" s="86" t="n"/>
-      <c r="E20" s="67" t="n"/>
-      <c r="F20" s="68" t="n"/>
-      <c r="G20" s="72" t="n"/>
-      <c r="H20" s="68" t="n"/>
-    </row>
-    <row r="21">
-      <c r="B21" s="70" t="n"/>
-      <c r="C21" s="67" t="n"/>
-      <c r="D21" s="86" t="n"/>
-      <c r="E21" s="67" t="n"/>
-      <c r="F21" s="68" t="n"/>
-      <c r="G21" s="72" t="n"/>
-      <c r="H21" s="68" t="n"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="70" t="n"/>
-      <c r="C22" s="67" t="n"/>
-      <c r="D22" s="86" t="n"/>
-      <c r="E22" s="67" t="n"/>
-      <c r="F22" s="68" t="n"/>
-      <c r="G22" s="72" t="n"/>
-      <c r="H22" s="68" t="n"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="70" t="n"/>
-      <c r="C23" s="67" t="n"/>
-      <c r="D23" s="86" t="n"/>
-      <c r="E23" s="67" t="n"/>
-      <c r="F23" s="68" t="n"/>
-      <c r="G23" s="72" t="n"/>
-      <c r="H23" s="68" t="n"/>
-    </row>
-    <row r="24">
-      <c r="B24" s="70" t="n"/>
-      <c r="C24" s="67" t="n"/>
-      <c r="D24" s="86" t="n"/>
-      <c r="E24" s="67" t="n"/>
-      <c r="F24" s="68" t="n"/>
-      <c r="G24" s="72" t="n"/>
-      <c r="H24" s="68" t="n"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="70" t="n"/>
-      <c r="C25" s="67" t="n"/>
-      <c r="D25" s="86" t="n"/>
-      <c r="E25" s="67" t="n"/>
-      <c r="F25" s="68" t="n"/>
-      <c r="G25" s="72" t="n"/>
-      <c r="H25" s="68" t="n"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="70" t="n"/>
-      <c r="C26" s="67" t="n"/>
-      <c r="D26" s="86" t="n"/>
-      <c r="E26" s="67" t="n"/>
-      <c r="F26" s="68" t="n"/>
-      <c r="G26" s="72" t="n"/>
-      <c r="H26" s="68" t="n"/>
-    </row>
-    <row r="27">
-      <c r="B27" s="70" t="n"/>
-      <c r="C27" s="67" t="n"/>
-      <c r="D27" s="86" t="n"/>
-      <c r="E27" s="67" t="n"/>
-      <c r="F27" s="68" t="n"/>
-      <c r="G27" s="72" t="n"/>
-      <c r="H27" s="68" t="n"/>
-    </row>
-    <row r="28">
-      <c r="B28" s="70" t="n"/>
-      <c r="C28" s="67" t="n"/>
-      <c r="D28" s="86" t="n"/>
-      <c r="E28" s="67" t="n"/>
-      <c r="F28" s="68" t="n"/>
-      <c r="G28" s="72" t="n"/>
-      <c r="H28" s="68" t="n"/>
-    </row>
-    <row r="29">
-      <c r="B29" s="70" t="n"/>
-      <c r="C29" s="67" t="n"/>
-      <c r="D29" s="86" t="n"/>
-      <c r="E29" s="67" t="n"/>
-      <c r="F29" s="68" t="n"/>
-      <c r="G29" s="72" t="n"/>
-      <c r="H29" s="68" t="n"/>
-    </row>
-    <row r="30">
-      <c r="B30" s="70" t="n"/>
-      <c r="C30" s="67" t="n"/>
-      <c r="D30" s="86" t="n"/>
-      <c r="E30" s="67" t="n"/>
-      <c r="F30" s="68" t="n"/>
-      <c r="G30" s="72" t="n"/>
-      <c r="H30" s="68" t="n"/>
-    </row>
-    <row r="31">
-      <c r="C31" s="67" t="n"/>
-      <c r="D31" s="86" t="n"/>
-      <c r="E31" s="67" t="n"/>
-      <c r="F31" s="68" t="n"/>
-      <c r="G31" s="72" t="n"/>
-      <c r="H31" s="68" t="n"/>
-    </row>
-    <row r="32">
-      <c r="C32" s="67" t="n"/>
-      <c r="D32" s="86" t="n"/>
-      <c r="E32" s="67" t="n"/>
-      <c r="F32" s="68" t="n"/>
-      <c r="G32" s="72" t="n"/>
-      <c r="H32" s="68" t="n"/>
-    </row>
-    <row r="33">
-      <c r="C33" s="67" t="n"/>
-      <c r="D33" s="86" t="n"/>
-      <c r="E33" s="67" t="n"/>
-      <c r="F33" s="68" t="n"/>
-      <c r="G33" s="72" t="n"/>
-      <c r="H33" s="68" t="n"/>
-    </row>
-    <row r="34">
-      <c r="C34" s="67" t="n"/>
-      <c r="D34" s="86" t="n"/>
-      <c r="E34" s="67" t="n"/>
-      <c r="F34" s="68" t="n"/>
-      <c r="G34" s="72" t="n"/>
-      <c r="H34" s="68" t="n"/>
-    </row>
-    <row r="35">
-      <c r="C35" s="67" t="n"/>
-      <c r="D35" s="86" t="n"/>
-      <c r="E35" s="67" t="n"/>
-      <c r="F35" s="68" t="n"/>
-      <c r="G35" s="72" t="n"/>
-      <c r="H35" s="68" t="n"/>
-    </row>
-    <row r="36">
-      <c r="C36" s="67" t="n"/>
-      <c r="D36" s="86" t="n"/>
-      <c r="E36" s="67" t="n"/>
-      <c r="F36" s="68" t="n"/>
-      <c r="G36" s="72" t="n"/>
-      <c r="H36" s="68" t="n"/>
-    </row>
-    <row r="37">
-      <c r="C37" s="67" t="n"/>
-      <c r="D37" s="86" t="n"/>
-      <c r="E37" s="67" t="n"/>
-      <c r="F37" s="68" t="n"/>
-      <c r="G37" s="72" t="n"/>
-      <c r="H37" s="68" t="n"/>
-    </row>
-    <row r="38">
-      <c r="C38" s="67" t="n"/>
-      <c r="D38" s="86" t="n"/>
-      <c r="E38" s="67" t="n"/>
-      <c r="F38" s="68" t="n"/>
-      <c r="G38" s="72" t="n"/>
-      <c r="H38" s="68" t="n"/>
-    </row>
-    <row r="39">
-      <c r="C39" s="67" t="n"/>
-      <c r="D39" s="86" t="n"/>
-      <c r="E39" s="67" t="n"/>
-      <c r="F39" s="68" t="n"/>
-      <c r="G39" s="72" t="n"/>
-      <c r="H39" s="68" t="n"/>
-    </row>
-    <row r="40">
-      <c r="C40" s="67" t="n"/>
-      <c r="D40" s="86" t="n"/>
-      <c r="E40" s="67" t="n"/>
-      <c r="F40" s="68" t="n"/>
-      <c r="G40" s="72" t="n"/>
-      <c r="H40" s="68" t="n"/>
-    </row>
-    <row r="41">
-      <c r="C41" s="67" t="n"/>
-      <c r="D41" s="86" t="n"/>
-      <c r="E41" s="67" t="n"/>
-      <c r="F41" s="68" t="n"/>
-      <c r="G41" s="72" t="n"/>
-      <c r="H41" s="68" t="n"/>
-    </row>
-    <row r="42">
-      <c r="C42" s="67" t="n"/>
-      <c r="D42" s="86" t="n"/>
-      <c r="E42" s="67" t="n"/>
-      <c r="F42" s="68" t="n"/>
-      <c r="G42" s="72" t="n"/>
-      <c r="H42" s="68" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6152,7 +5880,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6267,51 +5995,51 @@
         </is>
       </c>
       <c r="E11" s="43">
-        <f>ExFactory!G5</f>
+        <f>Demand!C34</f>
         <v/>
       </c>
       <c r="F11" s="43">
-        <f>ExFactory!G6</f>
+        <f>Demand!D34</f>
         <v/>
       </c>
       <c r="G11" s="43">
-        <f>ExFactory!G7</f>
+        <f>Demand!E34</f>
         <v/>
       </c>
       <c r="H11" s="43">
-        <f>ExFactory!G8</f>
+        <f>Demand!F34</f>
         <v/>
       </c>
       <c r="I11" s="43">
-        <f>ExFactory!G9</f>
+        <f>Demand!G34</f>
         <v/>
       </c>
       <c r="J11" s="43">
-        <f>ExFactory!G10</f>
+        <f>Demand!H34</f>
         <v/>
       </c>
       <c r="K11" s="43">
-        <f>ExFactory!G11</f>
+        <f>Demand!I34</f>
         <v/>
       </c>
       <c r="L11" s="43">
-        <f>ExFactory!G12</f>
+        <f>Demand!J34</f>
         <v/>
       </c>
       <c r="M11" s="43">
-        <f>ExFactory!G13</f>
+        <f>Demand!K34</f>
         <v/>
       </c>
       <c r="N11" s="43">
-        <f>ExFactory!G14</f>
+        <f>Demand!L34</f>
         <v/>
       </c>
       <c r="O11" s="43">
-        <f>ExFactory!G15</f>
+        <f>Demand!M34</f>
         <v/>
       </c>
       <c r="P11" s="43">
-        <f>ExFactory!G16</f>
+        <f>Demand!N34</f>
         <v/>
       </c>
       <c r="Q11" s="16">
@@ -7738,7 +7466,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Fix demand selector - all formulas now tie correctly
AUDIT FIXES:
- Unmerged cells B13:E13 that were blocking data write
- Fixed Scenario 1 data (row 13-14): Jan-Dec values now correct
- Fixed Scenario 2 formulas (row 17-22): proper formula chain
- Fixed Model column mapping: E→C, F→D, etc. (offset of 2)

FORMULA CHAIN NOW CORRECT:
- Selector C3=1 → pulls Demand rows 13-14 (Original Base)
- Selector C3=2 → pulls Demand rows 21-22 (BOD Nov 2025)

Scenario 2 chain: Scripts(17) × Comm%(18) = Total(19) × Coverage%(20) = Covered(21)
</commit_message>
<xml_diff>
--- a/Cardamyst Affordability Model - Final.xlsx
+++ b/Cardamyst Affordability Model - Final.xlsx
@@ -2236,51 +2236,51 @@
         </is>
       </c>
       <c r="E4" s="15">
+        <f>IF($C$3=1,Demand!C13,Demand!C21)</f>
+        <v/>
+      </c>
+      <c r="F4" s="15">
+        <f>IF($C$3=1,Demand!D13,Demand!D21)</f>
+        <v/>
+      </c>
+      <c r="G4" s="15">
         <f>IF($C$3=1,Demand!E13,Demand!E21)</f>
         <v/>
       </c>
-      <c r="F4" s="15">
+      <c r="H4" s="15">
         <f>IF($C$3=1,Demand!F13,Demand!F21)</f>
         <v/>
       </c>
-      <c r="G4" s="15">
+      <c r="I4" s="15">
         <f>IF($C$3=1,Demand!G13,Demand!G21)</f>
         <v/>
       </c>
-      <c r="H4" s="15">
+      <c r="J4" s="15">
         <f>IF($C$3=1,Demand!H13,Demand!H21)</f>
         <v/>
       </c>
-      <c r="I4" s="15">
+      <c r="K4" s="15">
         <f>IF($C$3=1,Demand!I13,Demand!I21)</f>
         <v/>
       </c>
-      <c r="J4" s="15">
+      <c r="L4" s="15">
         <f>IF($C$3=1,Demand!J13,Demand!J21)</f>
         <v/>
       </c>
-      <c r="K4" s="15">
+      <c r="M4" s="15">
         <f>IF($C$3=1,Demand!K13,Demand!K21)</f>
         <v/>
       </c>
-      <c r="L4" s="15">
+      <c r="N4" s="15">
         <f>IF($C$3=1,Demand!L13,Demand!L21)</f>
         <v/>
       </c>
-      <c r="M4" s="15">
+      <c r="O4" s="15">
         <f>IF($C$3=1,Demand!M13,Demand!M21)</f>
         <v/>
       </c>
-      <c r="N4" s="15">
+      <c r="P4" s="15">
         <f>IF($C$3=1,Demand!N13,Demand!N21)</f>
-        <v/>
-      </c>
-      <c r="O4" s="15">
-        <f>IF($C$3=1,Demand!O13,Demand!O21)</f>
-        <v/>
-      </c>
-      <c r="P4" s="15">
-        <f>IF($C$3=1,Demand!P13,Demand!P21)</f>
         <v/>
       </c>
       <c r="Q4" s="16">
@@ -2295,51 +2295,51 @@
         </is>
       </c>
       <c r="E5" s="15">
+        <f>IF($C$3=1,Demand!C14,Demand!C22)</f>
+        <v/>
+      </c>
+      <c r="F5" s="15">
+        <f>IF($C$3=1,Demand!D14,Demand!D22)</f>
+        <v/>
+      </c>
+      <c r="G5" s="15">
         <f>IF($C$3=1,Demand!E14,Demand!E22)</f>
         <v/>
       </c>
-      <c r="F5" s="15">
+      <c r="H5" s="15">
         <f>IF($C$3=1,Demand!F14,Demand!F22)</f>
         <v/>
       </c>
-      <c r="G5" s="15">
+      <c r="I5" s="15">
         <f>IF($C$3=1,Demand!G14,Demand!G22)</f>
         <v/>
       </c>
-      <c r="H5" s="15">
+      <c r="J5" s="15">
         <f>IF($C$3=1,Demand!H14,Demand!H22)</f>
         <v/>
       </c>
-      <c r="I5" s="15">
+      <c r="K5" s="15">
         <f>IF($C$3=1,Demand!I14,Demand!I22)</f>
         <v/>
       </c>
-      <c r="J5" s="15">
+      <c r="L5" s="15">
         <f>IF($C$3=1,Demand!J14,Demand!J22)</f>
         <v/>
       </c>
-      <c r="K5" s="15">
+      <c r="M5" s="15">
         <f>IF($C$3=1,Demand!K14,Demand!K22)</f>
         <v/>
       </c>
-      <c r="L5" s="15">
+      <c r="N5" s="15">
         <f>IF($C$3=1,Demand!L14,Demand!L22)</f>
         <v/>
       </c>
-      <c r="M5" s="15">
+      <c r="O5" s="15">
         <f>IF($C$3=1,Demand!M14,Demand!M22)</f>
         <v/>
       </c>
-      <c r="N5" s="15">
+      <c r="P5" s="15">
         <f>IF($C$3=1,Demand!N14,Demand!N22)</f>
-        <v/>
-      </c>
-      <c r="O5" s="15">
-        <f>IF($C$3=1,Demand!O14,Demand!O22)</f>
-        <v/>
-      </c>
-      <c r="P5" s="15">
-        <f>IF($C$3=1,Demand!P14,Demand!P22)</f>
         <v/>
       </c>
       <c r="Q5" s="16">
@@ -3979,6 +3979,15 @@
           <t>TRx Forecast (Covered Commercial)</t>
         </is>
       </c>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" t="n">
+        <v>50.23</v>
+      </c>
+      <c r="E13" t="n">
+        <v>83.78</v>
+      </c>
       <c r="F13" s="86" t="n">
         <v>131.82</v>
       </c>
@@ -4007,7 +4016,7 @@
         <v>3322.67</v>
       </c>
       <c r="O13" s="86">
-        <f>+SUM(C10:N10)</f>
+        <f>SUM(C13:N13)</f>
         <v/>
       </c>
     </row>
@@ -4054,7 +4063,7 @@
         <v>359.88</v>
       </c>
       <c r="O14" s="86">
-        <f>+SUM(C11:N11)</f>
+        <f>SUM(C14:N14)</f>
         <v/>
       </c>
     </row>
@@ -4140,7 +4149,7 @@
         <v>6813</v>
       </c>
       <c r="O17" s="86">
-        <f>+SUM(C14:N14)</f>
+        <f>SUM(C17:N17)</f>
         <v/>
       </c>
     </row>
@@ -4152,51 +4161,51 @@
         </is>
       </c>
       <c r="C18" s="63">
-        <f>+Assumptions!C50</f>
+        <f>Assumptions!C50</f>
         <v/>
       </c>
       <c r="D18" s="63">
-        <f>+Assumptions!C51</f>
+        <f>Assumptions!C51</f>
         <v/>
       </c>
       <c r="E18" s="63">
-        <f>+Assumptions!C52</f>
+        <f>Assumptions!C52</f>
         <v/>
       </c>
       <c r="F18" s="63">
-        <f>+Assumptions!C53</f>
+        <f>Assumptions!C53</f>
         <v/>
       </c>
       <c r="G18" s="63">
-        <f>+Assumptions!C54</f>
+        <f>Assumptions!C54</f>
         <v/>
       </c>
       <c r="H18" s="63">
-        <f>+Assumptions!C55</f>
+        <f>Assumptions!C55</f>
         <v/>
       </c>
       <c r="I18" s="63">
-        <f>+Assumptions!C56</f>
+        <f>Assumptions!C56</f>
         <v/>
       </c>
       <c r="J18" s="63">
-        <f>+Assumptions!C57</f>
+        <f>Assumptions!C57</f>
         <v/>
       </c>
       <c r="K18" s="63">
-        <f>+Assumptions!C58</f>
+        <f>Assumptions!C58</f>
         <v/>
       </c>
       <c r="L18" s="63">
-        <f>+Assumptions!C59</f>
+        <f>Assumptions!C59</f>
         <v/>
       </c>
       <c r="M18" s="63">
-        <f>+Assumptions!C60</f>
+        <f>Assumptions!C60</f>
         <v/>
       </c>
       <c r="N18" s="63">
-        <f>+Assumptions!C61</f>
+        <f>Assumptions!C61</f>
         <v/>
       </c>
       <c r="O18" s="86" t="n"/>
@@ -4209,55 +4218,55 @@
         </is>
       </c>
       <c r="C19" s="86">
-        <f>+C14*C15</f>
+        <f>C17*C18</f>
         <v/>
       </c>
       <c r="D19" s="86">
-        <f>+D14*D15</f>
+        <f>D17*D18</f>
         <v/>
       </c>
       <c r="E19" s="86">
-        <f>+E14*E15</f>
+        <f>E17*E18</f>
         <v/>
       </c>
       <c r="F19" s="86">
-        <f>+F14*F15</f>
+        <f>F17*F18</f>
         <v/>
       </c>
       <c r="G19" s="86">
-        <f>+G14*G15</f>
+        <f>G17*G18</f>
         <v/>
       </c>
       <c r="H19" s="86">
-        <f>+H14*H15</f>
+        <f>H17*H18</f>
         <v/>
       </c>
       <c r="I19" s="86">
-        <f>+I14*I15</f>
+        <f>I17*I18</f>
         <v/>
       </c>
       <c r="J19" s="86">
-        <f>+J14*J15</f>
+        <f>J17*J18</f>
         <v/>
       </c>
       <c r="K19" s="86">
-        <f>+K14*K15</f>
+        <f>K17*K18</f>
         <v/>
       </c>
       <c r="L19" s="86">
-        <f>+L14*L15</f>
+        <f>L17*L18</f>
         <v/>
       </c>
       <c r="M19" s="86">
-        <f>+M14*M15</f>
+        <f>M17*M18</f>
         <v/>
       </c>
       <c r="N19" s="86">
-        <f>+N14*N15</f>
+        <f>N17*N18</f>
         <v/>
       </c>
       <c r="O19" s="86">
-        <f>+SUM(C16:N16)</f>
+        <f>SUM(C19:N19)</f>
         <v/>
       </c>
     </row>
@@ -4269,51 +4278,51 @@
         </is>
       </c>
       <c r="C20" s="63">
-        <f>+Assumptions!C22</f>
+        <f>Assumptions!C22</f>
         <v/>
       </c>
       <c r="D20" s="63">
-        <f>+Assumptions!C23</f>
+        <f>Assumptions!C23</f>
         <v/>
       </c>
       <c r="E20" s="63">
-        <f>+Assumptions!C24</f>
+        <f>Assumptions!C24</f>
         <v/>
       </c>
       <c r="F20" s="63">
-        <f>+Assumptions!C25</f>
+        <f>Assumptions!C25</f>
         <v/>
       </c>
       <c r="G20" s="63">
-        <f>+Assumptions!C26</f>
+        <f>Assumptions!C26</f>
         <v/>
       </c>
       <c r="H20" s="63">
-        <f>+Assumptions!C27</f>
+        <f>Assumptions!C27</f>
         <v/>
       </c>
       <c r="I20" s="63">
-        <f>+Assumptions!C28</f>
+        <f>Assumptions!C28</f>
         <v/>
       </c>
       <c r="J20" s="63">
-        <f>+Assumptions!C29</f>
+        <f>Assumptions!C29</f>
         <v/>
       </c>
       <c r="K20" s="63">
-        <f>+Assumptions!C30</f>
+        <f>Assumptions!C30</f>
         <v/>
       </c>
       <c r="L20" s="63">
-        <f>+Assumptions!C31</f>
+        <f>Assumptions!C31</f>
         <v/>
       </c>
       <c r="M20" s="63">
-        <f>+Assumptions!C32</f>
+        <f>Assumptions!C32</f>
         <v/>
       </c>
       <c r="N20" s="63">
-        <f>+Assumptions!C33</f>
+        <f>Assumptions!C33</f>
         <v/>
       </c>
       <c r="O20" s="86" t="n"/>
@@ -4325,55 +4334,55 @@
         </is>
       </c>
       <c r="C21" s="86">
-        <f>+C16*C17</f>
+        <f>C19*C20</f>
         <v/>
       </c>
       <c r="D21" s="86">
-        <f>+D16*D17</f>
+        <f>D19*D20</f>
         <v/>
       </c>
       <c r="E21" s="86">
-        <f>+E16*E17</f>
+        <f>E19*E20</f>
         <v/>
       </c>
       <c r="F21" s="86">
-        <f>+F16*F17</f>
+        <f>F19*F20</f>
         <v/>
       </c>
       <c r="G21" s="86">
-        <f>+G16*G17</f>
+        <f>G19*G20</f>
         <v/>
       </c>
       <c r="H21" s="86">
-        <f>+H16*H17</f>
+        <f>H19*H20</f>
         <v/>
       </c>
       <c r="I21" s="86">
-        <f>+I16*I17</f>
+        <f>I19*I20</f>
         <v/>
       </c>
       <c r="J21" s="86">
-        <f>+J16*J17</f>
+        <f>J19*J20</f>
         <v/>
       </c>
       <c r="K21" s="86">
-        <f>+K16*K17</f>
+        <f>K19*K20</f>
         <v/>
       </c>
       <c r="L21" s="86">
-        <f>+L16*L17</f>
+        <f>L19*L20</f>
         <v/>
       </c>
       <c r="M21" s="86">
-        <f>+M16*M17</f>
+        <f>M19*M20</f>
         <v/>
       </c>
       <c r="N21" s="86">
-        <f>+N16*N17</f>
+        <f>N19*N20</f>
         <v/>
       </c>
       <c r="O21" s="86">
-        <f>+SUM(C18:N18)</f>
+        <f>SUM(C21:N21)</f>
         <v/>
       </c>
     </row>
@@ -4384,55 +4393,55 @@
         </is>
       </c>
       <c r="C22" s="86">
-        <f>+C16-C18</f>
+        <f>C19-C21</f>
         <v/>
       </c>
       <c r="D22" s="86">
-        <f>+D16-D18</f>
+        <f>D19-D21</f>
         <v/>
       </c>
       <c r="E22" s="86">
-        <f>+E16-E18</f>
+        <f>E19-E21</f>
         <v/>
       </c>
       <c r="F22" s="86">
-        <f>+F16-F18</f>
+        <f>F19-F21</f>
         <v/>
       </c>
       <c r="G22" s="86">
-        <f>+G16-G18</f>
+        <f>G19-G21</f>
         <v/>
       </c>
       <c r="H22" s="86">
-        <f>+H16-H18</f>
+        <f>H19-H21</f>
         <v/>
       </c>
       <c r="I22" s="86">
-        <f>+I16-I18</f>
+        <f>I19-I21</f>
         <v/>
       </c>
       <c r="J22" s="86">
-        <f>+J16-J18</f>
+        <f>J19-J21</f>
         <v/>
       </c>
       <c r="K22" s="86">
-        <f>+K16-K18</f>
+        <f>K19-K21</f>
         <v/>
       </c>
       <c r="L22" s="86">
-        <f>+L16-L18</f>
+        <f>L19-L21</f>
         <v/>
       </c>
       <c r="M22" s="86">
-        <f>+M16-M18</f>
+        <f>M19-M21</f>
         <v/>
       </c>
       <c r="N22" s="86">
-        <f>+N16-N18</f>
+        <f>N19-N21</f>
         <v/>
       </c>
       <c r="O22" s="86">
-        <f>+SUM(C19:N19)</f>
+        <f>SUM(C22:N22)</f>
         <v/>
       </c>
     </row>
@@ -4858,9 +4867,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A24:F24"/>
-    <mergeCell ref="B13:E13"/>
+  <mergeCells count="2">
     <mergeCell ref="B8:E8"/>
     <mergeCell ref="A4:F4"/>
   </mergeCells>

</xml_diff>